<commit_message>
walk through F2, F3, the volcano supplement and the QC supplement
</commit_message>
<xml_diff>
--- a/05_Figures/HRvLR/F3_People/c_data/f3_people.xlsx
+++ b/05_Figures/HRvLR/F3_People/c_data/f3_people.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11924" uniqueCount="4098">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11957" uniqueCount="4119">
   <si>
     <t>sheet</t>
   </si>
@@ -303,7 +303,7 @@
     <t>best single feature per task</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/06_Classification/01_Proteins/c_data/protein_classification.xlsx</t>
+    <t>03_Group_comparisons/HRvLR/05_Classification/01_Proteins/c_data/protein_classification.xlsx</t>
   </si>
   <si>
     <t>auc, counts</t>
@@ -318,7 +318,7 @@
     <t>group difference against continuous interaction</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/07_Trait_Associations/c_data/trait_associations.xlsx</t>
+    <t>03_Group_comparisons/HRvLR/06_Trait_Associations/c_data/trait_associations.xlsx</t>
   </si>
   <si>
     <t>group_difference; interaction</t>
@@ -11886,25 +11886,25 @@
     <t>LR_S30</t>
   </si>
   <si>
-    <t>b01ac1f6d6d70cf871c6751d533234fd</t>
-  </si>
-  <si>
-    <t>02_HRvLR_groups/06_Classification/02_Sets/c_data/set_classification.xlsx</t>
-  </si>
-  <si>
-    <t>2d5c57240ac4c245f6b3ae6409d38693</t>
-  </si>
-  <si>
-    <t>02_HRvLR_groups/06_Classification/03_Modules/c_data/module_classification.xlsx</t>
-  </si>
-  <si>
-    <t>3160dbe9810c780b4924a19c1e8f2f4f</t>
+    <t>a95402d461edffdb1bfe52e24fa7f7f5</t>
+  </si>
+  <si>
+    <t>03_Group_comparisons/HRvLR/05_Classification/02_Sets/c_data/set_classification.xlsx</t>
+  </si>
+  <si>
+    <t>b178395b3633ca781c3d08c789b73be2</t>
+  </si>
+  <si>
+    <t>03_Group_comparisons/HRvLR/05_Classification/03_Modules/c_data/module_classification.xlsx</t>
+  </si>
+  <si>
+    <t>40af5ef3d827e7eda16199768c84b50c</t>
   </si>
   <si>
     <t>associate</t>
   </si>
   <si>
-    <t>9ac893e6ae1926d745c3c47a1bb5b588</t>
+    <t>22366981c91de546cdab366e3b1baab4</t>
   </si>
   <si>
     <t>continuous</t>
@@ -11913,7 +11913,7 @@
     <t>04_Continuous_no_group/01_Trait_Associations/01_Proteins/c_data/protein_trait_associations.xlsx</t>
   </si>
   <si>
-    <t>400e71a7f9b28b71965d7d0a160d06c9</t>
+    <t>4c94a3c340f52458c17e5a5394bde99d</t>
   </si>
   <si>
     <t>corrected</t>
@@ -11928,7 +11928,7 @@
     <t>phenotype</t>
   </si>
   <si>
-    <t>00_Input/phenotype.csv</t>
+    <t>00_Setup/Input/phenotype.csv</t>
   </si>
   <si>
     <t>5a1989db406daa0b70189a9f0df52cf3</t>
@@ -12036,12 +12036,24 @@
     <t>1.2.1</t>
   </si>
   <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
+  </si>
+  <si>
     <t>farver</t>
   </si>
   <si>
     <t>2.1.2</t>
   </si>
   <si>
+    <t>fastmap</t>
+  </si>
+  <si>
+    <t>1.2.0</t>
+  </si>
+  <si>
     <t>foreach</t>
   </si>
   <si>
@@ -12105,6 +12117,18 @@
     <t>1.1.4</t>
   </si>
   <si>
+    <t>htmltools</t>
+  </si>
+  <si>
+    <t>0.5.9</t>
+  </si>
+  <si>
+    <t>htmlwidgets</t>
+  </si>
+  <si>
+    <t>1.6.4</t>
+  </si>
+  <si>
     <t>IRanges</t>
   </si>
   <si>
@@ -12117,6 +12141,18 @@
     <t>1.0.14</t>
   </si>
   <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
+    <t>knitr</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
     <t>labeling</t>
   </si>
   <si>
@@ -12132,9 +12168,6 @@
     <t>lifecycle</t>
   </si>
   <si>
-    <t>1.0.5</t>
-  </si>
-  <si>
     <t>magrittr</t>
   </si>
   <si>
@@ -12165,6 +12198,12 @@
     <t>3.1-169</t>
   </si>
   <si>
+    <t>otel</t>
+  </si>
+  <si>
+    <t>0.2.0</t>
+  </si>
+  <si>
     <t>patchwork</t>
   </si>
   <si>
@@ -12246,6 +12285,12 @@
     <t>CRAN (R 4.6.1)</t>
   </si>
   <si>
+    <t>rmarkdown</t>
+  </si>
+  <si>
+    <t>2.31</t>
+  </si>
+  <si>
     <t>rprojroot</t>
   </si>
   <si>
@@ -12312,6 +12357,12 @@
     <t>0.5.0</t>
   </si>
   <si>
+    <t>utf8</t>
+  </si>
+  <si>
+    <t>1.2.6</t>
+  </si>
+  <si>
     <t>vctrs</t>
   </si>
   <si>
@@ -12328,6 +12379,18 @@
   </si>
   <si>
     <t>3.0.2</t>
+  </si>
+  <si>
+    <t>xfun</t>
+  </si>
+  <si>
+    <t>0.57</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -101862,7 +101925,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -102134,7 +102197,7 @@
         <v>4014</v>
       </c>
       <c r="B25" t="s">
-        <v>4005</v>
+        <v>4015</v>
       </c>
       <c r="C25" t="s">
         <v>3971</v>
@@ -102142,10 +102205,10 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>4015</v>
+        <v>4016</v>
       </c>
       <c r="B26" t="s">
-        <v>4016</v>
+        <v>4017</v>
       </c>
       <c r="C26" t="s">
         <v>3971</v>
@@ -102153,10 +102216,10 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>4017</v>
+        <v>4018</v>
       </c>
       <c r="B27" t="s">
-        <v>4018</v>
+        <v>4009</v>
       </c>
       <c r="C27" t="s">
         <v>3971</v>
@@ -102192,7 +102255,7 @@
         <v>4024</v>
       </c>
       <c r="C30" t="s">
-        <v>3968</v>
+        <v>3971</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -102236,7 +102299,7 @@
         <v>4032</v>
       </c>
       <c r="C34" t="s">
-        <v>3971</v>
+        <v>3968</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -102299,7 +102362,7 @@
         <v>4043</v>
       </c>
       <c r="B40" t="s">
-        <v>4044</v>
+        <v>4001</v>
       </c>
       <c r="C40" t="s">
         <v>3971</v>
@@ -102307,10 +102370,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
+        <v>4044</v>
+      </c>
+      <c r="B41" t="s">
         <v>4045</v>
-      </c>
-      <c r="B41" t="s">
-        <v>4046</v>
       </c>
       <c r="C41" t="s">
         <v>3971</v>
@@ -102318,10 +102381,10 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
+        <v>4046</v>
+      </c>
+      <c r="B42" t="s">
         <v>4047</v>
-      </c>
-      <c r="B42" t="s">
-        <v>4048</v>
       </c>
       <c r="C42" t="s">
         <v>3971</v>
@@ -102329,10 +102392,10 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
+        <v>4048</v>
+      </c>
+      <c r="B43" t="s">
         <v>4049</v>
-      </c>
-      <c r="B43" t="s">
-        <v>4050</v>
       </c>
       <c r="C43" t="s">
         <v>3971</v>
@@ -102340,10 +102403,10 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
+        <v>4050</v>
+      </c>
+      <c r="B44" t="s">
         <v>4051</v>
-      </c>
-      <c r="B44" t="s">
-        <v>4052</v>
       </c>
       <c r="C44" t="s">
         <v>3971</v>
@@ -102351,10 +102414,10 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
+        <v>4052</v>
+      </c>
+      <c r="B45" t="s">
         <v>4053</v>
-      </c>
-      <c r="B45" t="s">
-        <v>4054</v>
       </c>
       <c r="C45" t="s">
         <v>3971</v>
@@ -102362,10 +102425,10 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
+        <v>4054</v>
+      </c>
+      <c r="B46" t="s">
         <v>4055</v>
-      </c>
-      <c r="B46" t="s">
-        <v>4056</v>
       </c>
       <c r="C46" t="s">
         <v>3971</v>
@@ -102373,10 +102436,10 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
+        <v>4056</v>
+      </c>
+      <c r="B47" t="s">
         <v>4057</v>
-      </c>
-      <c r="B47" t="s">
-        <v>4058</v>
       </c>
       <c r="C47" t="s">
         <v>3971</v>
@@ -102384,10 +102447,10 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
+        <v>4058</v>
+      </c>
+      <c r="B48" t="s">
         <v>4059</v>
-      </c>
-      <c r="B48" t="s">
-        <v>4060</v>
       </c>
       <c r="C48" t="s">
         <v>3971</v>
@@ -102395,10 +102458,10 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
+        <v>4060</v>
+      </c>
+      <c r="B49" t="s">
         <v>4061</v>
-      </c>
-      <c r="B49" t="s">
-        <v>4062</v>
       </c>
       <c r="C49" t="s">
         <v>3971</v>
@@ -102406,10 +102469,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
+        <v>4062</v>
+      </c>
+      <c r="B50" t="s">
         <v>4063</v>
-      </c>
-      <c r="B50" t="s">
-        <v>4064</v>
       </c>
       <c r="C50" t="s">
         <v>3971</v>
@@ -102417,10 +102480,10 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
+        <v>4064</v>
+      </c>
+      <c r="B51" t="s">
         <v>4065</v>
-      </c>
-      <c r="B51" t="s">
-        <v>4066</v>
       </c>
       <c r="C51" t="s">
         <v>3971</v>
@@ -102428,21 +102491,21 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
+        <v>4066</v>
+      </c>
+      <c r="B52" t="s">
         <v>4067</v>
       </c>
-      <c r="B52" t="s">
-        <v>4068</v>
-      </c>
       <c r="C52" t="s">
-        <v>4069</v>
+        <v>3971</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>4070</v>
+        <v>4068</v>
       </c>
       <c r="B53" t="s">
-        <v>4071</v>
+        <v>4069</v>
       </c>
       <c r="C53" t="s">
         <v>3971</v>
@@ -102450,21 +102513,21 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>4072</v>
+        <v>4070</v>
       </c>
       <c r="B54" t="s">
-        <v>4073</v>
+        <v>4071</v>
       </c>
       <c r="C54" t="s">
-        <v>3968</v>
+        <v>3971</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>4074</v>
+        <v>4072</v>
       </c>
       <c r="B55" t="s">
-        <v>4075</v>
+        <v>4073</v>
       </c>
       <c r="C55" t="s">
         <v>3971</v>
@@ -102472,10 +102535,10 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>4076</v>
+        <v>4074</v>
       </c>
       <c r="B56" t="s">
-        <v>4077</v>
+        <v>4075</v>
       </c>
       <c r="C56" t="s">
         <v>3971</v>
@@ -102483,10 +102546,10 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>4078</v>
+        <v>4076</v>
       </c>
       <c r="B57" t="s">
-        <v>4079</v>
+        <v>4077</v>
       </c>
       <c r="C57" t="s">
         <v>3971</v>
@@ -102494,10 +102557,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>4080</v>
+        <v>4078</v>
       </c>
       <c r="B58" t="s">
-        <v>4081</v>
+        <v>4079</v>
       </c>
       <c r="C58" t="s">
         <v>3971</v>
@@ -102505,21 +102568,21 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
+        <v>4080</v>
+      </c>
+      <c r="B59" t="s">
+        <v>4081</v>
+      </c>
+      <c r="C59" t="s">
         <v>4082</v>
-      </c>
-      <c r="B59" t="s">
-        <v>4083</v>
-      </c>
-      <c r="C59" t="s">
-        <v>3971</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
+        <v>4083</v>
+      </c>
+      <c r="B60" t="s">
         <v>4084</v>
-      </c>
-      <c r="B60" t="s">
-        <v>4085</v>
       </c>
       <c r="C60" t="s">
         <v>3971</v>
@@ -102527,10 +102590,10 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
+        <v>4085</v>
+      </c>
+      <c r="B61" t="s">
         <v>4086</v>
-      </c>
-      <c r="B61" t="s">
-        <v>4087</v>
       </c>
       <c r="C61" t="s">
         <v>3971</v>
@@ -102538,13 +102601,13 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
+        <v>4087</v>
+      </c>
+      <c r="B62" t="s">
         <v>4088</v>
       </c>
-      <c r="B62" t="s">
-        <v>4044</v>
-      </c>
       <c r="C62" t="s">
-        <v>3971</v>
+        <v>3968</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -102552,7 +102615,7 @@
         <v>4089</v>
       </c>
       <c r="B63" t="s">
-        <v>3999</v>
+        <v>4090</v>
       </c>
       <c r="C63" t="s">
         <v>3971</v>
@@ -102560,10 +102623,10 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>4090</v>
+        <v>4091</v>
       </c>
       <c r="B64" t="s">
-        <v>4091</v>
+        <v>4092</v>
       </c>
       <c r="C64" t="s">
         <v>3971</v>
@@ -102571,10 +102634,10 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>4092</v>
+        <v>4093</v>
       </c>
       <c r="B65" t="s">
-        <v>4093</v>
+        <v>4094</v>
       </c>
       <c r="C65" t="s">
         <v>3971</v>
@@ -102582,10 +102645,10 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>4094</v>
+        <v>4095</v>
       </c>
       <c r="B66" t="s">
-        <v>4095</v>
+        <v>4096</v>
       </c>
       <c r="C66" t="s">
         <v>3971</v>
@@ -102593,12 +102656,133 @@
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>4096</v>
+        <v>4097</v>
       </c>
       <c r="B67" t="s">
-        <v>4097</v>
+        <v>4098</v>
       </c>
       <c r="C67" t="s">
+        <v>3971</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
+        <v>4099</v>
+      </c>
+      <c r="B68" t="s">
+        <v>4100</v>
+      </c>
+      <c r="C68" t="s">
+        <v>3971</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
+        <v>4101</v>
+      </c>
+      <c r="B69" t="s">
+        <v>4102</v>
+      </c>
+      <c r="C69" t="s">
+        <v>3971</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
+        <v>4103</v>
+      </c>
+      <c r="B70" t="s">
+        <v>4057</v>
+      </c>
+      <c r="C70" t="s">
+        <v>3971</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
+        <v>4104</v>
+      </c>
+      <c r="B71" t="s">
+        <v>3999</v>
+      </c>
+      <c r="C71" t="s">
+        <v>3971</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" t="s">
+        <v>4105</v>
+      </c>
+      <c r="B72" t="s">
+        <v>4106</v>
+      </c>
+      <c r="C72" t="s">
+        <v>3971</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" t="s">
+        <v>4107</v>
+      </c>
+      <c r="B73" t="s">
+        <v>4108</v>
+      </c>
+      <c r="C73" t="s">
+        <v>3971</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" t="s">
+        <v>4109</v>
+      </c>
+      <c r="B74" t="s">
+        <v>4110</v>
+      </c>
+      <c r="C74" t="s">
+        <v>3971</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" t="s">
+        <v>4111</v>
+      </c>
+      <c r="B75" t="s">
+        <v>4112</v>
+      </c>
+      <c r="C75" t="s">
+        <v>3971</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" t="s">
+        <v>4113</v>
+      </c>
+      <c r="B76" t="s">
+        <v>4114</v>
+      </c>
+      <c r="C76" t="s">
+        <v>3971</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" t="s">
+        <v>4115</v>
+      </c>
+      <c r="B77" t="s">
+        <v>4116</v>
+      </c>
+      <c r="C77" t="s">
+        <v>3971</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" t="s">
+        <v>4117</v>
+      </c>
+      <c r="B78" t="s">
+        <v>4118</v>
+      </c>
+      <c r="C78" t="s">
         <v>3971</v>
       </c>
     </row>

</xml_diff>